<commit_message>
Created UI and made UI test excel driven
</commit_message>
<xml_diff>
--- a/DownloadedExcels/dsrProfileData (1).xlsx
+++ b/DownloadedExcels/dsrProfileData (1).xlsx
@@ -83220,27 +83220,27 @@
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>COL10036</t>
+          <t>COL10022</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>order booker 817</t>
+          <t>AUTODSR_68E63</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>21312312720</t>
+          <t>03115314900</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>0001</t>
+          <t>0002</t>
         </is>
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t/>
+          <t>EMP335004</t>
         </is>
       </c>
       <c r="G548" t="inlineStr">
@@ -83255,7 +83255,7 @@
       </c>
       <c r="I548" t="inlineStr">
         <is>
-          <t>2025-03-12</t>
+          <t>2025-02-26</t>
         </is>
       </c>
       <c r="J548" t="inlineStr">
@@ -83280,7 +83280,7 @@
       </c>
       <c r="N548" t="inlineStr">
         <is>
-          <t/>
+          <t>Smith_DM</t>
         </is>
       </c>
       <c r="O548" t="inlineStr">
@@ -83300,7 +83300,7 @@
       </c>
       <c r="R548" t="inlineStr">
         <is>
-          <t>ads</t>
+          <t>asd</t>
         </is>
       </c>
       <c r="S548" t="inlineStr">
@@ -83325,7 +83325,7 @@
       </c>
       <c r="W548" t="inlineStr">
         <is>
-          <t>22222221122</t>
+          <t>21421212133</t>
         </is>
       </c>
       <c r="X548" t="inlineStr">
@@ -83340,17 +83340,17 @@
       </c>
       <c r="Z548" t="inlineStr">
         <is>
-          <t>22321321212111213</t>
+          <t>43030222448759162</t>
         </is>
       </c>
       <c r="AA548" t="inlineStr">
         <is>
-          <t>2025-03-12</t>
+          <t>2025-02-26</t>
         </is>
       </c>
       <c r="AB548" t="inlineStr">
         <is>
-          <t>2025-03-27</t>
+          <t>2025-02-28</t>
         </is>
       </c>
       <c r="AC548" t="inlineStr">
@@ -83360,7 +83360,7 @@
       </c>
       <c r="AD548" t="inlineStr">
         <is>
-          <t/>
+          <t>AUTODSR_776E6</t>
         </is>
       </c>
     </row>
@@ -83372,27 +83372,27 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>COL10022</t>
+          <t>COL10036</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>AUTODSR_EDC72</t>
+          <t>order booker 817</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
         <is>
-          <t>03026779100</t>
+          <t>21312312720</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>0002</t>
+          <t>0001</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
         <is>
-          <t>EMP335004</t>
+          <t/>
         </is>
       </c>
       <c r="G549" t="inlineStr">
@@ -83407,7 +83407,7 @@
       </c>
       <c r="I549" t="inlineStr">
         <is>
-          <t>2025-02-26</t>
+          <t>2025-03-12</t>
         </is>
       </c>
       <c r="J549" t="inlineStr">
@@ -83432,7 +83432,7 @@
       </c>
       <c r="N549" t="inlineStr">
         <is>
-          <t>Smith_DM</t>
+          <t/>
         </is>
       </c>
       <c r="O549" t="inlineStr">
@@ -83452,7 +83452,7 @@
       </c>
       <c r="R549" t="inlineStr">
         <is>
-          <t>asd</t>
+          <t>ads</t>
         </is>
       </c>
       <c r="S549" t="inlineStr">
@@ -83477,7 +83477,7 @@
       </c>
       <c r="W549" t="inlineStr">
         <is>
-          <t>21421212133</t>
+          <t>22222221122</t>
         </is>
       </c>
       <c r="X549" t="inlineStr">
@@ -83492,17 +83492,17 @@
       </c>
       <c r="Z549" t="inlineStr">
         <is>
-          <t>88474990598050162</t>
+          <t>22321321212111213</t>
         </is>
       </c>
       <c r="AA549" t="inlineStr">
         <is>
-          <t>2025-02-26</t>
+          <t>2025-03-12</t>
         </is>
       </c>
       <c r="AB549" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2025-03-27</t>
         </is>
       </c>
       <c r="AC549" t="inlineStr">
@@ -83512,7 +83512,7 @@
       </c>
       <c r="AD549" t="inlineStr">
         <is>
-          <t>AUTODSR_776E6</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -84593,12 +84593,12 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>AUTODSR_69E70</t>
+          <t>AUTODSR_F6F7B</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>03028547300</t>
+          <t>03116663200</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
@@ -84708,7 +84708,7 @@
       </c>
       <c r="Z557" t="inlineStr">
         <is>
-          <t>50413033627981279</t>
+          <t>94546049933001596</t>
         </is>
       </c>
       <c r="AA557" t="inlineStr">

</xml_diff>